<commit_message>
Update consistency dataset and table retrieval optimization
</commit_message>
<xml_diff>
--- a/法規資料_md_clean_leaf_json/evaluation_dataset/consistency_qa.xlsx
+++ b/法規資料_md_clean_leaf_json/evaluation_dataset/consistency_qa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruby0\Desktop\EY\legal-rag-workflow-main\08_leaf_json_embedding_問答\法規資料_md_clean_leaf_json\evaluation_dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877216FD-8D95-4BD9-B658-206844A8F0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD77483-4C7D-4540-9E7A-5B815C3FC1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8360" yWindow="0" windowWidth="10860" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -96,9 +96,6 @@
     <t>C001_Q03</t>
   </si>
   <si>
-    <t>內部控制包含哪三種因素？</t>
-  </si>
-  <si>
     <t>C002_Q01</t>
   </si>
   <si>
@@ -192,9 +189,6 @@
     <t>C004_Q03</t>
   </si>
   <si>
-    <t>資訊服務包含哪五種服務型態？</t>
-  </si>
-  <si>
     <t>C005_Q01</t>
   </si>
   <si>
@@ -226,13 +220,21 @@
   </si>
   <si>
     <t>採用靜態密碼進行身分驗證時，公司應進行妥善處理，代表密碼連續錯了幾次？</t>
+  </si>
+  <si>
+    <t>內部控制制度設計時，應納入哪些主要控制因素？</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>資訊服務包含哪三種服務型態？</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +272,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="4">
@@ -341,7 +350,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -369,6 +378,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -668,7 +683,7 @@
     <col min="11" max="11" width="15.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" ht="42">
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="28">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -782,8 +797,8 @@
       <c r="D4" s="6">
         <v>3</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>23</v>
+      <c r="E4" s="11" t="s">
+        <v>65</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>15</v>
@@ -804,10 +819,10 @@
     </row>
     <row r="5" spans="1:11" ht="84">
       <c r="A5" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>24</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>25</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>13</v>
@@ -816,19 +831,19 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>26</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>27</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="H5" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="9" t="s">
         <v>28</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>29</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>19</v>
@@ -837,10 +852,10 @@
     </row>
     <row r="6" spans="1:11" ht="84">
       <c r="A6" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>13</v>
@@ -849,19 +864,19 @@
         <v>2</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>16</v>
       </c>
       <c r="H6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>29</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>19</v>
@@ -870,10 +885,10 @@
     </row>
     <row r="7" spans="1:11" ht="84">
       <c r="A7" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>13</v>
@@ -882,19 +897,19 @@
         <v>3</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>16</v>
       </c>
       <c r="H7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="9" t="s">
         <v>28</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>29</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>19</v>
@@ -903,10 +918,10 @@
     </row>
     <row r="8" spans="1:11" ht="112">
       <c r="A8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>35</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>13</v>
@@ -915,19 +930,19 @@
         <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>19</v>
@@ -936,10 +951,10 @@
     </row>
     <row r="9" spans="1:11" ht="112">
       <c r="A9" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>13</v>
@@ -948,19 +963,19 @@
         <v>2</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F9" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>39</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>40</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>19</v>
@@ -969,10 +984,10 @@
     </row>
     <row r="10" spans="1:11" ht="112">
       <c r="A10" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>13</v>
@@ -981,19 +996,19 @@
         <v>3</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>19</v>
@@ -1002,10 +1017,10 @@
     </row>
     <row r="11" spans="1:11" ht="70">
       <c r="A11" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>45</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>46</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>13</v>
@@ -1014,19 +1029,19 @@
         <v>1</v>
       </c>
       <c r="E11" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="I11" s="9" t="s">
         <v>50</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>51</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>19</v>
@@ -1035,10 +1050,10 @@
     </row>
     <row r="12" spans="1:11" ht="70">
       <c r="A12" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>13</v>
@@ -1047,19 +1062,19 @@
         <v>2</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>51</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>19</v>
@@ -1068,10 +1083,10 @@
     </row>
     <row r="13" spans="1:11" ht="70">
       <c r="A13" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>13</v>
@@ -1079,20 +1094,20 @@
       <c r="D13" s="9">
         <v>3</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>55</v>
+      <c r="E13" s="12" t="s">
+        <v>66</v>
       </c>
       <c r="F13" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="H13" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="I13" s="9" t="s">
         <v>50</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>51</v>
       </c>
       <c r="J13" s="9" t="s">
         <v>19</v>
@@ -1101,10 +1116,10 @@
     </row>
     <row r="14" spans="1:11" ht="70">
       <c r="A14" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>13</v>
@@ -1113,31 +1128,31 @@
         <v>1</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="J14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" ht="56">
+      <c r="A15" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="I14" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K14" s="7"/>
-    </row>
-    <row r="15" spans="1:11" ht="70">
-      <c r="A15" s="8" t="s">
-        <v>63</v>
-      </c>
       <c r="B15" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>13</v>
@@ -1146,19 +1161,19 @@
         <v>2</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F15" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="I15" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>62</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>19</v>
@@ -1167,10 +1182,10 @@
     </row>
     <row r="16" spans="1:11" ht="70">
       <c r="A16" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>13</v>
@@ -1179,19 +1194,19 @@
         <v>3</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F16" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="I16" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>19</v>

</xml_diff>